<commit_message>
Add Airtable Files Downloader module to main CLI. Introduce functionality for downloading PDF files from Airtable CSV exports, including user prompts for file paths and options for dry-run and limiting downloads. Update main menu to include the new feature and enhance README documentation for usage instructions. Add pandas and tqdm dependencies for CSV processing and progress tracking.
</commit_message>
<xml_diff>
--- a/scripts/generate_report_from_webgains/enriched_webgains_reports/Transacciones_newcop_2509_enriched.xlsx
+++ b/scripts/generate_report_from_webgains/enriched_webgains_reports/Transacciones_newcop_2509_enriched.xlsx
@@ -860,7 +860,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Essentials Hoodie (FW22) Light Oatmeal</t>
+          <t>Adidas Samba OG Maroon Off White Gum</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -875,7 +875,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Adidas Samba OG Maroon Off White Gum</t>
+          <t>Essentials Hoodie (FW22) Light Oatmeal</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
@@ -965,7 +965,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Adidas Adizero Evo SL White Pure Teal</t>
+          <t>Puma Arizona SD Flat Bronze-Alpine Snow</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
@@ -980,7 +980,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Puma Arizona SD Flat Bronze-Alpine Snow</t>
+          <t>Essentials Pullover Hoodie (FW22) Stretch Limo/Black</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
@@ -995,7 +995,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Essentials Pullover Hoodie (FW22) Stretch Limo/Black</t>
+          <t>Adidas Adizero Evo SL White Pure Teal</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
@@ -1085,7 +1085,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Air Force 1 Rope Laces Black</t>
+          <t>Air Jordan 4 Retro OG SP Undefeated</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
@@ -1100,7 +1100,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Retro OG SP Undefeated</t>
+          <t>Air Force 1 Rope Laces Black</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
@@ -1419,22 +1419,22 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>127.5</v>
+        <v>70</v>
       </c>
       <c r="C2" s="13" t="n">
-        <v>7.65</v>
+        <v>4.2</v>
       </c>
       <c r="D2" s="13" t="n">
-        <v>2.3</v>
+        <v>1.26</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>09/30/25 16:25</t>
+          <t>09/30/25 12:49</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>79375</t>
+          <t>79361</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1454,17 +1454,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Adidas Adizero Evo SL White Pure Teal</t>
+          <t>Puma Arizona SD Flat Bronze-Alpine Snow</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>42 EU - 8.5 US</t>
+          <t>37 EU - 5 US</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>JS4487</t>
+          <t>402362-04</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1485,24 +1485,20 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>protomela@yahoo.es</t>
+          <t>sandra.isla.88@gmail.com</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Jose luis</t>
+          <t>Sandra</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Sanchis mañanos</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>+34671639303</t>
-        </is>
-      </c>
+          <t>Isla</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
           <t>First Order</t>
@@ -1540,26 +1536,26 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Digital Expand</t>
+          <t>Mathias Kraft</t>
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>4.2</v>
+        <v>10.8</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>1.26</v>
+        <v>3.24</v>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>09/30/25 12:49</t>
+          <t>09/30/25 15:30</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>79361</t>
+          <t>79365</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
@@ -1579,17 +1575,17 @@
       </c>
       <c r="J3" s="15" t="inlineStr">
         <is>
-          <t>Puma Arizona SD Flat Bronze-Alpine Snow</t>
+          <t>Essentials Pullover Hoodie (FW22) Stretch Limo/Black</t>
         </is>
       </c>
       <c r="K3" s="15" t="inlineStr">
         <is>
-          <t>37 EU - 5 US</t>
+          <t>M</t>
         </is>
       </c>
       <c r="L3" s="15" t="inlineStr">
         <is>
-          <t>402362-04</t>
+          <t>192BT212110F</t>
         </is>
       </c>
       <c r="M3" s="15" t="inlineStr">
@@ -1610,28 +1606,32 @@
       <c r="P3" s="15" t="inlineStr"/>
       <c r="Q3" s="15" t="inlineStr">
         <is>
-          <t>sandra.isla.88@gmail.com</t>
+          <t>gaizkablanco7@gmail.com</t>
         </is>
       </c>
       <c r="R3" s="15" t="inlineStr">
         <is>
-          <t>Sandra</t>
+          <t>Gaizka</t>
         </is>
       </c>
       <c r="S3" s="15" t="inlineStr">
         <is>
-          <t>Isla</t>
-        </is>
-      </c>
-      <c r="T3" s="15" t="inlineStr"/>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="T3" s="15" t="inlineStr">
+        <is>
+          <t>+34664564676</t>
+        </is>
+      </c>
       <c r="U3" s="15" t="inlineStr">
         <is>
-          <t>First Order</t>
+          <t>Repeat Customer (Order #3)</t>
         </is>
       </c>
       <c r="V3" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="W3" s="15" t="inlineStr">
@@ -1639,21 +1639,9 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X3" s="15" t="inlineStr">
-        <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="Y3" s="15" t="inlineStr">
-        <is>
-          <t>cpc</t>
-        </is>
-      </c>
-      <c r="Z3" s="15" t="inlineStr">
-        <is>
-          <t>{campaignname}</t>
-        </is>
-      </c>
+      <c r="X3" s="15" t="inlineStr"/>
+      <c r="Y3" s="15" t="inlineStr"/>
+      <c r="Z3" s="15" t="inlineStr"/>
       <c r="AA3" s="15" t="inlineStr"/>
       <c r="AB3" s="15" t="inlineStr"/>
       <c r="AC3" s="15" t="inlineStr"/>
@@ -1661,26 +1649,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mathias Kraft</t>
+          <t>Digital Expand</t>
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>180</v>
+        <v>127.5</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>10.8</v>
+        <v>7.65</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>3.24</v>
+        <v>2.3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>09/30/25 15:30</t>
+          <t>09/30/25 16:25</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>79365</t>
+          <t>79375</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1700,17 +1688,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Essentials Pullover Hoodie (FW22) Stretch Limo/Black</t>
+          <t>Adidas Adizero Evo SL White Pure Teal</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>42 EU - 8.5 US</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>192BT212110F</t>
+          <t>JS4487</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1731,32 +1719,32 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>gaizkablanco7@gmail.com</t>
+          <t>protomela@yahoo.es</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Gaizka</t>
+          <t>Jose luis</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Blanco</t>
+          <t>Sanchis mañanos</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>+34664564676</t>
+          <t>+34671639303</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Repeat Customer (Order #3)</t>
+          <t>First Order</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -1764,9 +1752,21 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>cpc</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>{campaignname}</t>
+        </is>
+      </c>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
@@ -2117,31 +2117,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Webravo SRL</t>
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>330</v>
+        <v>110</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>19.8</v>
+        <v>6.6</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>5.94</v>
+        <v>1.98</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>09/24/25 14:24</t>
+          <t>09/22/25 20:03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>78891</t>
+          <t>78812</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2156,17 +2156,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Denim Tears The Cotton Wreath Sweatshirt Black</t>
+          <t>Adidas Samba OG Maroon Off White Gum</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>39.3 EU - 6.5 US</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>DENIMBW</t>
+          <t>JR8844</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -2187,17 +2187,17 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>sandionisio7@gmail.com</t>
+          <t>ccarbonell.torrees@gmail.com</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Antonio</t>
+          <t>Carlota</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Neira Parra</t>
+          <t>Carbonell Torres</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -2216,9 +2216,21 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>cpc</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>{campaignname}</t>
+        </is>
+      </c>
       <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
@@ -2472,31 +2484,31 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Webravo SRL</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>110</v>
+        <v>330</v>
       </c>
       <c r="C11" s="16" t="n">
-        <v>6.6</v>
+        <v>19.8</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>1.98</v>
+        <v>5.94</v>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>09/22/25 20:03</t>
+          <t>09/24/25 14:24</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>78812</t>
+          <t>78891</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -2511,17 +2523,17 @@
       </c>
       <c r="J11" s="15" t="inlineStr">
         <is>
-          <t>Adidas Samba OG Maroon Off White Gum</t>
+          <t>Denim Tears The Cotton Wreath Sweatshirt Black</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>39.3 EU - 6.5 US</t>
+          <t>M</t>
         </is>
       </c>
       <c r="L11" s="15" t="inlineStr">
         <is>
-          <t>JR8844</t>
+          <t>DENIMBW</t>
         </is>
       </c>
       <c r="M11" s="15" t="inlineStr">
@@ -2542,17 +2554,17 @@
       <c r="P11" s="15" t="inlineStr"/>
       <c r="Q11" s="15" t="inlineStr">
         <is>
-          <t>ccarbonell.torrees@gmail.com</t>
+          <t>sandionisio7@gmail.com</t>
         </is>
       </c>
       <c r="R11" s="15" t="inlineStr">
         <is>
-          <t>Carlota</t>
+          <t>Antonio</t>
         </is>
       </c>
       <c r="S11" s="15" t="inlineStr">
         <is>
-          <t>Carbonell Torres</t>
+          <t>Neira Parra</t>
         </is>
       </c>
       <c r="T11" s="15" t="inlineStr"/>
@@ -2571,21 +2583,9 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X11" s="15" t="inlineStr">
-        <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="Y11" s="15" t="inlineStr">
-        <is>
-          <t>cpc</t>
-        </is>
-      </c>
-      <c r="Z11" s="15" t="inlineStr">
-        <is>
-          <t>{campaignname}</t>
-        </is>
-      </c>
+      <c r="X11" s="15" t="inlineStr"/>
+      <c r="Y11" s="15" t="inlineStr"/>
+      <c r="Z11" s="15" t="inlineStr"/>
       <c r="AA11" s="15" t="inlineStr"/>
       <c r="AB11" s="15" t="inlineStr"/>
       <c r="AC11" s="15" t="inlineStr"/>
@@ -2593,26 +2593,26 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Purplee Corp</t>
+          <t>Invoke AB</t>
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>170</v>
+        <v>350</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>10.2</v>
+        <v>21</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>3.06</v>
+        <v>6.3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>09/22/25 14:45</t>
+          <t>09/20/25 11:34</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6903116824917</t>
+          <t>6900010221909</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2632,17 +2632,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Air Force 1 Rope Laces Black</t>
+          <t>Air Jordan 4 Retro OG SP Undefeated</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>45 EU - 11 US</t>
+          <t>46 EU - 12 US</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>CW2288-001-BLACK</t>
+          <t>IB1519-200</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -2663,54 +2663,38 @@
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>am.nieto.ro@gmail.com</t>
+          <t>blanco_negro1977@hotmail.com</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Ana María</t>
+          <t>Jorge</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Nieto Rodríguez</t>
+          <t>Lozano lozano</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>+34650261577</t>
+          <t>+34654624273</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>First Order</t>
+          <t>Repeat Customer (Order #4)</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>cpc</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>{campaignname}</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
@@ -2718,26 +2702,26 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Digital Expand</t>
+          <t>Purplee Corp</t>
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>6</v>
+        <v>10.2</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>1.8</v>
+        <v>3.06</v>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>09/18/25 19:39</t>
+          <t>09/22/25 14:45</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>6897694179669</t>
+          <t>6903116824917</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -2747,27 +2731,27 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr">
         <is>
-          <t>Puma Speedcat TTF Dark Chocolate Frosted Ivory</t>
+          <t>Air Force 1 Rope Laces Black</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>37 EU - 4.5 US</t>
+          <t>45 EU - 11 US</t>
         </is>
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
-          <t>403903-01</t>
+          <t>CW2288-001-BLACK</t>
         </is>
       </c>
       <c r="M13" s="15" t="inlineStr">
@@ -2788,20 +2772,24 @@
       <c r="P13" s="15" t="inlineStr"/>
       <c r="Q13" s="15" t="inlineStr">
         <is>
-          <t>albertolagoalba@gmail.com</t>
+          <t>am.nieto.ro@gmail.com</t>
         </is>
       </c>
       <c r="R13" s="15" t="inlineStr">
         <is>
-          <t>Alberto</t>
+          <t>Ana María</t>
         </is>
       </c>
       <c r="S13" s="15" t="inlineStr">
         <is>
-          <t>Lago alba</t>
-        </is>
-      </c>
-      <c r="T13" s="15" t="inlineStr"/>
+          <t>Nieto Rodríguez</t>
+        </is>
+      </c>
+      <c r="T13" s="15" t="inlineStr">
+        <is>
+          <t>+34650261577</t>
+        </is>
+      </c>
       <c r="U13" s="15" t="inlineStr">
         <is>
           <t>First Order</t>
@@ -2817,9 +2805,21 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X13" s="15" t="inlineStr"/>
-      <c r="Y13" s="15" t="inlineStr"/>
-      <c r="Z13" s="15" t="inlineStr"/>
+      <c r="X13" s="15" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="Y13" s="15" t="inlineStr">
+        <is>
+          <t>cpc</t>
+        </is>
+      </c>
+      <c r="Z13" s="15" t="inlineStr">
+        <is>
+          <t>{campaignname}</t>
+        </is>
+      </c>
       <c r="AA13" s="15" t="inlineStr"/>
       <c r="AB13" s="15" t="inlineStr"/>
       <c r="AC13" s="15" t="inlineStr"/>
@@ -2827,26 +2827,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Invoke AB</t>
+          <t>Digital Expand</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>350</v>
+        <v>120</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>6.3</v>
+        <v>1.8</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>09/20/25 11:34</t>
+          <t>09/18/25 19:39</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>6900010221909</t>
+          <t>6897694179669</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2856,27 +2856,27 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Air Jordan 4 Retro OG SP Undefeated</t>
+          <t>Puma Speedcat TTF Dark Chocolate Frosted Ivory</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>46 EU - 12 US</t>
+          <t>37 EU - 4.5 US</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IB1519-200</t>
+          <t>403903-01</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2897,35 +2897,35 @@
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>blanco_negro1977@hotmail.com</t>
+          <t>albertolagoalba@gmail.com</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Jorge</t>
+          <t>Alberto</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Lozano lozano</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>+34654624273</t>
-        </is>
-      </c>
+          <t>Lago alba</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Repeat Customer (Order #4)</t>
+          <t>First Order</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
@@ -2936,26 +2936,26 @@
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Pashion.dk ApS</t>
         </is>
       </c>
       <c r="B15" s="16" t="n">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="C15" s="16" t="n">
-        <v>6.6</v>
+        <v>14</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>1.98</v>
+        <v>4.2</v>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>09/19/25 23:39</t>
+          <t>09/16/25 20:51</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>78602</t>
+          <t>6894848966997</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
@@ -2965,27 +2965,27 @@
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="J15" s="15" t="inlineStr">
         <is>
-          <t>Adidas Samba OG Maroon Off White Gum</t>
+          <t>Air Jordan 3 Retro Black Cat</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>40.6 EU - 7.5 US</t>
+          <t>36.5 EU - 4.5 US</t>
         </is>
       </c>
       <c r="L15" s="15" t="inlineStr">
         <is>
-          <t>JR8844</t>
+          <t>CT8532-001</t>
         </is>
       </c>
       <c r="M15" s="15" t="inlineStr">
@@ -3006,28 +3006,32 @@
       <c r="P15" s="15" t="inlineStr"/>
       <c r="Q15" s="15" t="inlineStr">
         <is>
-          <t>anamariamenzr1@hotmail.com</t>
+          <t>restauracionespablogarcia@hotmail.com</t>
         </is>
       </c>
       <c r="R15" s="15" t="inlineStr">
         <is>
-          <t>Ana</t>
+          <t>Lorena</t>
         </is>
       </c>
       <c r="S15" s="15" t="inlineStr">
         <is>
-          <t>Menezo Rojas</t>
-        </is>
-      </c>
-      <c r="T15" s="15" t="inlineStr"/>
+          <t>Liaño cobo</t>
+        </is>
+      </c>
+      <c r="T15" s="15" t="inlineStr">
+        <is>
+          <t>+34699813897</t>
+        </is>
+      </c>
       <c r="U15" s="15" t="inlineStr">
         <is>
-          <t>First Order</t>
+          <t>Repeat Customer (Order #2)</t>
         </is>
       </c>
       <c r="V15" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W15" s="15" t="inlineStr">
@@ -3035,21 +3039,9 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X15" s="15" t="inlineStr">
-        <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="Y15" s="15" t="inlineStr">
-        <is>
-          <t>cpc</t>
-        </is>
-      </c>
-      <c r="Z15" s="15" t="inlineStr">
-        <is>
-          <t>{campaignname}</t>
-        </is>
-      </c>
+      <c r="X15" s="15" t="inlineStr"/>
+      <c r="Y15" s="15" t="inlineStr"/>
+      <c r="Z15" s="15" t="inlineStr"/>
       <c r="AA15" s="15" t="inlineStr"/>
       <c r="AB15" s="15" t="inlineStr"/>
       <c r="AC15" s="15" t="inlineStr"/>
@@ -3057,26 +3049,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Webravo SRL</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1.62</v>
+        <v>1.98</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>09/20/25 11:53</t>
+          <t>09/19/25 23:39</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>78608</t>
+          <t>78602</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3096,17 +3088,17 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Adidas Samba Jane Cream Black Gum</t>
+          <t>Adidas Samba OG Maroon Off White Gum</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>38 EU - 5.5 US</t>
+          <t>40.6 EU - 7.5 US</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>JR7338</t>
+          <t>JR8844</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -3127,17 +3119,17 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>paulalopezpuyol12@gmail.com</t>
+          <t>anamariamenzr1@hotmail.com</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Paula</t>
+          <t>Ana</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>López Puyol</t>
+          <t>Menezo Rojas</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -3178,26 +3170,26 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Pashion.dk ApS</t>
+          <t>Webravo SRL</t>
         </is>
       </c>
       <c r="B17" s="16" t="n">
-        <v>280</v>
+        <v>90</v>
       </c>
       <c r="C17" s="16" t="n">
-        <v>14</v>
+        <v>5.4</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>4.2</v>
+        <v>1.62</v>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>09/16/25 20:51</t>
+          <t>09/20/25 11:53</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>6894848966997</t>
+          <t>78608</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -3207,27 +3199,27 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="J17" s="15" t="inlineStr">
         <is>
-          <t>Air Jordan 3 Retro Black Cat</t>
+          <t>Adidas Samba Jane Cream Black Gum</t>
         </is>
       </c>
       <c r="K17" s="15" t="inlineStr">
         <is>
-          <t>36.5 EU - 4.5 US</t>
+          <t>38 EU - 5.5 US</t>
         </is>
       </c>
       <c r="L17" s="15" t="inlineStr">
         <is>
-          <t>CT8532-001</t>
+          <t>JR7338</t>
         </is>
       </c>
       <c r="M17" s="15" t="inlineStr">
@@ -3248,32 +3240,28 @@
       <c r="P17" s="15" t="inlineStr"/>
       <c r="Q17" s="15" t="inlineStr">
         <is>
-          <t>restauracionespablogarcia@hotmail.com</t>
+          <t>paulalopezpuyol12@gmail.com</t>
         </is>
       </c>
       <c r="R17" s="15" t="inlineStr">
         <is>
-          <t>Lorena</t>
+          <t>Paula</t>
         </is>
       </c>
       <c r="S17" s="15" t="inlineStr">
         <is>
-          <t>Liaño cobo</t>
-        </is>
-      </c>
-      <c r="T17" s="15" t="inlineStr">
-        <is>
-          <t>+34699813897</t>
-        </is>
-      </c>
+          <t>López Puyol</t>
+        </is>
+      </c>
+      <c r="T17" s="15" t="inlineStr"/>
       <c r="U17" s="15" t="inlineStr">
         <is>
-          <t>Repeat Customer (Order #2)</t>
+          <t>First Order</t>
         </is>
       </c>
       <c r="V17" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W17" s="15" t="inlineStr">
@@ -3281,9 +3269,21 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X17" s="15" t="inlineStr"/>
-      <c r="Y17" s="15" t="inlineStr"/>
-      <c r="Z17" s="15" t="inlineStr"/>
+      <c r="X17" s="15" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="Y17" s="15" t="inlineStr">
+        <is>
+          <t>cpc</t>
+        </is>
+      </c>
+      <c r="Z17" s="15" t="inlineStr">
+        <is>
+          <t>{campaignname}</t>
+        </is>
+      </c>
       <c r="AA17" s="15" t="inlineStr"/>
       <c r="AB17" s="15" t="inlineStr"/>
       <c r="AC17" s="15" t="inlineStr"/>
@@ -3400,26 +3400,26 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Pashion.dk ApS</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B19" s="16" t="n">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="C19" s="16" t="n">
-        <v>6</v>
+        <v>5.28</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>1.8</v>
+        <v>1.58</v>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>09/16/25 16:05</t>
+          <t>09/15/25 11:50</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>78437</t>
+          <t>78383</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
@@ -3429,27 +3429,27 @@
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I19" s="17" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="J19" s="15" t="inlineStr">
         <is>
-          <t>Puma LaMelo Ball LaFrancé Amour Moment</t>
+          <t>Puma Speedcat OG Haute Coffee Frosted Ivory</t>
         </is>
       </c>
       <c r="K19" s="15" t="inlineStr">
         <is>
-          <t>41 EU - 8.5 US</t>
+          <t>37 EU - 5 US</t>
         </is>
       </c>
       <c r="L19" s="15" t="inlineStr">
         <is>
-          <t>310864-01</t>
+          <t>398846-31</t>
         </is>
       </c>
       <c r="M19" s="15" t="inlineStr">
@@ -3470,32 +3470,28 @@
       <c r="P19" s="15" t="inlineStr"/>
       <c r="Q19" s="15" t="inlineStr">
         <is>
-          <t>alfredirriak24@gmail.com</t>
+          <t>ilargi-betea22@hotmail.com</t>
         </is>
       </c>
       <c r="R19" s="15" t="inlineStr">
         <is>
-          <t>Alfredo Dueñas</t>
+          <t>Elisabet</t>
         </is>
       </c>
       <c r="S19" s="15" t="inlineStr">
         <is>
-          <t>Fernández</t>
-        </is>
-      </c>
-      <c r="T19" s="15" t="inlineStr">
-        <is>
-          <t>+34613250693</t>
-        </is>
-      </c>
+          <t>Menen</t>
+        </is>
+      </c>
+      <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="15" t="inlineStr">
         <is>
-          <t>Repeat Customer (Order #2)</t>
+          <t>First Order</t>
         </is>
       </c>
       <c r="V19" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W19" s="15" t="inlineStr">
@@ -3503,21 +3499,9 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X19" s="15" t="inlineStr">
-        <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="Y19" s="15" t="inlineStr">
-        <is>
-          <t>cpc</t>
-        </is>
-      </c>
-      <c r="Z19" s="15" t="inlineStr">
-        <is>
-          <t>20498453736</t>
-        </is>
-      </c>
+      <c r="X19" s="15" t="inlineStr"/>
+      <c r="Y19" s="15" t="inlineStr"/>
+      <c r="Z19" s="15" t="inlineStr"/>
       <c r="AA19" s="15" t="inlineStr"/>
       <c r="AB19" s="15" t="inlineStr"/>
       <c r="AC19" s="15" t="inlineStr"/>
@@ -3634,26 +3618,26 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Pashion.dk ApS</t>
         </is>
       </c>
       <c r="B21" s="16" t="n">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="C21" s="16" t="n">
-        <v>5.28</v>
+        <v>6</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>1.58</v>
+        <v>1.8</v>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>09/15/25 11:50</t>
+          <t>09/16/25 16:05</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>78383</t>
+          <t>78437</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
@@ -3663,27 +3647,27 @@
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="J21" s="15" t="inlineStr">
         <is>
-          <t>Puma Speedcat OG Haute Coffee Frosted Ivory</t>
+          <t>Puma LaMelo Ball LaFrancé Amour Moment</t>
         </is>
       </c>
       <c r="K21" s="15" t="inlineStr">
         <is>
-          <t>37 EU - 5 US</t>
+          <t>41 EU - 8.5 US</t>
         </is>
       </c>
       <c r="L21" s="15" t="inlineStr">
         <is>
-          <t>398846-31</t>
+          <t>310864-01</t>
         </is>
       </c>
       <c r="M21" s="15" t="inlineStr">
@@ -3704,28 +3688,32 @@
       <c r="P21" s="15" t="inlineStr"/>
       <c r="Q21" s="15" t="inlineStr">
         <is>
-          <t>ilargi-betea22@hotmail.com</t>
+          <t>alfredirriak24@gmail.com</t>
         </is>
       </c>
       <c r="R21" s="15" t="inlineStr">
         <is>
-          <t>Elisabet</t>
+          <t>Alfredo Dueñas</t>
         </is>
       </c>
       <c r="S21" s="15" t="inlineStr">
         <is>
-          <t>Menen</t>
-        </is>
-      </c>
-      <c r="T21" s="15" t="inlineStr"/>
+          <t>Fernández</t>
+        </is>
+      </c>
+      <c r="T21" s="15" t="inlineStr">
+        <is>
+          <t>+34613250693</t>
+        </is>
+      </c>
       <c r="U21" s="15" t="inlineStr">
         <is>
-          <t>First Order</t>
+          <t>Repeat Customer (Order #2)</t>
         </is>
       </c>
       <c r="V21" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W21" s="15" t="inlineStr">
@@ -3733,9 +3721,21 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X21" s="15" t="inlineStr"/>
-      <c r="Y21" s="15" t="inlineStr"/>
-      <c r="Z21" s="15" t="inlineStr"/>
+      <c r="X21" s="15" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="Y21" s="15" t="inlineStr">
+        <is>
+          <t>cpc</t>
+        </is>
+      </c>
+      <c r="Z21" s="15" t="inlineStr">
+        <is>
+          <t>20498453736</t>
+        </is>
+      </c>
       <c r="AA21" s="15" t="inlineStr"/>
       <c r="AB21" s="15" t="inlineStr"/>
       <c r="AC21" s="15" t="inlineStr"/>
@@ -3743,26 +3743,26 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pashion.dk ApS</t>
+          <t>Purplee Corp</t>
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>120</v>
+        <v>82.5</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>6</v>
+        <v>4.95</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>1.8</v>
+        <v>1.49</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>09/15/25 11:46</t>
+          <t>09/14/25 12:50</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>78382</t>
+          <t>6891134681429</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3772,27 +3772,27 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Puma Speedcat TTF Dark Chocolate Frosted Ivory</t>
+          <t>Adidas Handball Spezial Core Black Pink</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>41 EU - 8 US</t>
+          <t>43.3 EU - 9.5 US</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>403903-01</t>
+          <t>IE5897</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -3813,24 +3813,20 @@
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>luiscompostizo@gmail.com</t>
+          <t>Slwoffi@hotmail.com</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Luis</t>
+          <t>Sonia</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Compostizo Garcia</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>+34722237884</t>
-        </is>
-      </c>
+          <t>Lwoff Ivanissevich</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr">
         <is>
           <t>First Order</t>
@@ -3841,16 +3837,8 @@
           <t>1</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>webgains</t>
-        </is>
-      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
@@ -3860,26 +3848,26 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Pashion.dk ApS</t>
         </is>
       </c>
       <c r="B23" s="16" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="C23" s="16" t="n">
-        <v>5.76</v>
+        <v>6</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>1.73</v>
+        <v>1.8</v>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>09/14/25 22:07</t>
+          <t>09/15/25 11:46</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>78374</t>
+          <t>78382</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
@@ -3889,27 +3877,27 @@
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="J23" s="15" t="inlineStr">
         <is>
-          <t>Adidas Samba OG Core Black</t>
+          <t>Puma Speedcat TTF Dark Chocolate Frosted Ivory</t>
         </is>
       </c>
       <c r="K23" s="15" t="inlineStr">
         <is>
-          <t>42.6 EU - 9 US</t>
+          <t>41 EU - 8 US</t>
         </is>
       </c>
       <c r="L23" s="15" t="inlineStr">
         <is>
-          <t>B75807</t>
+          <t>403903-01</t>
         </is>
       </c>
       <c r="M23" s="15" t="inlineStr">
@@ -3930,20 +3918,24 @@
       <c r="P23" s="15" t="inlineStr"/>
       <c r="Q23" s="15" t="inlineStr">
         <is>
-          <t>ydorgambide@gmail.com</t>
+          <t>luiscompostizo@gmail.com</t>
         </is>
       </c>
       <c r="R23" s="15" t="inlineStr">
         <is>
-          <t>Yago</t>
+          <t>Luis</t>
         </is>
       </c>
       <c r="S23" s="15" t="inlineStr">
         <is>
-          <t>Dorgambide Dios</t>
-        </is>
-      </c>
-      <c r="T23" s="15" t="inlineStr"/>
+          <t>Compostizo Garcia</t>
+        </is>
+      </c>
+      <c r="T23" s="15" t="inlineStr">
+        <is>
+          <t>+34722237884</t>
+        </is>
+      </c>
       <c r="U23" s="15" t="inlineStr">
         <is>
           <t>First Order</t>
@@ -3959,7 +3951,11 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="X23" s="15" t="inlineStr"/>
+      <c r="X23" s="15" t="inlineStr">
+        <is>
+          <t>webgains</t>
+        </is>
+      </c>
       <c r="Y23" s="15" t="inlineStr"/>
       <c r="Z23" s="15" t="inlineStr"/>
       <c r="AA23" s="15" t="inlineStr"/>
@@ -3969,26 +3965,26 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Purplee Corp</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>82.5</v>
+        <v>96</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>4.95</v>
+        <v>5.76</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>1.49</v>
+        <v>1.73</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>09/14/25 12:50</t>
+          <t>09/14/25 22:07</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>6891134681429</t>
+          <t>78374</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -4008,17 +4004,17 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Adidas Handball Spezial Core Black Pink</t>
+          <t>Adidas Samba OG Core Black</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>43.3 EU - 9.5 US</t>
+          <t>42.6 EU - 9 US</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>IE5897</t>
+          <t>B75807</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -4039,17 +4035,17 @@
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Slwoffi@hotmail.com</t>
+          <t>ydorgambide@gmail.com</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Sonia</t>
+          <t>Yago</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Lwoff Ivanissevich</t>
+          <t>Dorgambide Dios</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -4063,7 +4059,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="W24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
@@ -4074,26 +4074,26 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Digital Expand</t>
         </is>
       </c>
       <c r="B25" s="16" t="n">
-        <v>750</v>
+        <v>550</v>
       </c>
       <c r="C25" s="16" t="n">
-        <v>37.5</v>
+        <v>27.5</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>11.25</v>
+        <v>8.25</v>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>09/13/25 10:43</t>
+          <t>09/11/25 16:14</t>
         </is>
       </c>
       <c r="F25" s="15" t="inlineStr">
         <is>
-          <t>78157</t>
+          <t>6887025475925</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">
@@ -4113,17 +4113,17 @@
       </c>
       <c r="J25" s="15" t="inlineStr">
         <is>
-          <t>Dunk Low Off-White Lot 21</t>
+          <t>Air Jordan 1 Retro Low OG SP Travis Scott Velvet Brown</t>
         </is>
       </c>
       <c r="K25" s="15" t="inlineStr">
         <is>
-          <t>44 EU - 10 US</t>
+          <t>42 EU - 8.5 US</t>
         </is>
       </c>
       <c r="L25" s="15" t="inlineStr">
         <is>
-          <t>DM1602-100</t>
+          <t>DM7866-202</t>
         </is>
       </c>
       <c r="M25" s="15" t="inlineStr">
@@ -4144,28 +4144,32 @@
       <c r="P25" s="15" t="inlineStr"/>
       <c r="Q25" s="15" t="inlineStr">
         <is>
-          <t>juudith.rg@gmail.com</t>
+          <t>cristiancampos26500@gmail.com</t>
         </is>
       </c>
       <c r="R25" s="15" t="inlineStr">
         <is>
-          <t>Judith</t>
+          <t>Cristian</t>
         </is>
       </c>
       <c r="S25" s="15" t="inlineStr">
         <is>
-          <t>Robles Garcia</t>
-        </is>
-      </c>
-      <c r="T25" s="15" t="inlineStr"/>
+          <t>Campos Mata</t>
+        </is>
+      </c>
+      <c r="T25" s="15" t="inlineStr">
+        <is>
+          <t>+34632623867</t>
+        </is>
+      </c>
       <c r="U25" s="15" t="inlineStr">
         <is>
-          <t>First Order</t>
+          <t>Repeat Customer (Order #2)</t>
         </is>
       </c>
       <c r="V25" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W25" s="15" t="inlineStr">
@@ -4183,26 +4187,26 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Digital Expand</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>550</v>
+        <v>750</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>27.5</v>
+        <v>37.5</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>8.25</v>
+        <v>11.25</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>09/11/25 16:14</t>
+          <t>09/13/25 10:43</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>6887025475925</t>
+          <t>78157</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -4222,17 +4226,17 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Retro Low OG SP Travis Scott Velvet Brown</t>
+          <t>Dunk Low Off-White Lot 21</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>42 EU - 8.5 US</t>
+          <t>44 EU - 10 US</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>DM7866-202</t>
+          <t>DM1602-100</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -4253,32 +4257,28 @@
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>cristiancampos26500@gmail.com</t>
+          <t>juudith.rg@gmail.com</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Cristian</t>
+          <t>Judith</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Campos Mata</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>+34632623867</t>
-        </is>
-      </c>
+          <t>Robles Garcia</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Repeat Customer (Order #2)</t>
+          <t>First Order</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
@@ -4538,26 +4538,26 @@
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>Klarna Bank AB UK Branch</t>
+          <t>LINKGAINS PTE.LTD.</t>
         </is>
       </c>
       <c r="B29" s="16" t="n">
-        <v>153</v>
+        <v>335</v>
       </c>
       <c r="C29" s="16" t="n">
-        <v>7.65</v>
+        <v>16.75</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>2.3</v>
+        <v>5.03</v>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>09/10/25 09:03</t>
+          <t>09/09/25 17:32</t>
         </is>
       </c>
       <c r="F29" s="15" t="inlineStr">
         <is>
-          <t>77873</t>
+          <t>77821</t>
         </is>
       </c>
       <c r="G29" s="15" t="inlineStr">
@@ -4577,17 +4577,17 @@
       </c>
       <c r="J29" s="15" t="inlineStr">
         <is>
-          <t>Air Force 1 Rope Laces</t>
+          <t>ASICS Gel-NYC Cream Arctic Sky</t>
         </is>
       </c>
       <c r="K29" s="15" t="inlineStr">
         <is>
-          <t>38 EU - 5.5 US</t>
+          <t>40 EU - 7 US</t>
         </is>
       </c>
       <c r="L29" s="15" t="inlineStr">
         <is>
-          <t>CW2288-111ME</t>
+          <t>1203A383-107</t>
         </is>
       </c>
       <c r="M29" s="15" t="inlineStr">
@@ -4608,17 +4608,17 @@
       <c r="P29" s="15" t="inlineStr"/>
       <c r="Q29" s="15" t="inlineStr">
         <is>
-          <t>kaaa-95@hotmail.com</t>
+          <t>gestoriapradillo@gmail.com</t>
         </is>
       </c>
       <c r="R29" s="15" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>LAURA</t>
         </is>
       </c>
       <c r="S29" s="15" t="inlineStr">
         <is>
-          <t>Serrano Sánchez</t>
+          <t>BORRAJO ROMERO</t>
         </is>
       </c>
       <c r="T29" s="15" t="inlineStr"/>
@@ -4634,16 +4634,24 @@
       </c>
       <c r="W29" s="15" t="inlineStr">
         <is>
-          <t>an unknown source</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="X29" s="15" t="inlineStr">
         <is>
-          <t>webgains</t>
-        </is>
-      </c>
-      <c r="Y29" s="15" t="inlineStr"/>
-      <c r="Z29" s="15" t="inlineStr"/>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="Y29" s="15" t="inlineStr">
+        <is>
+          <t>cpc</t>
+        </is>
+      </c>
+      <c r="Z29" s="15" t="inlineStr">
+        <is>
+          <t>21366334315</t>
+        </is>
+      </c>
       <c r="AA29" s="15" t="inlineStr"/>
       <c r="AB29" s="15" t="inlineStr"/>
       <c r="AC29" s="15" t="inlineStr"/>
@@ -4651,26 +4659,26 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LINKGAINS PTE.LTD.</t>
+          <t>Klarna Bank AB UK Branch</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>335</v>
+        <v>153</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>16.75</v>
+        <v>7.65</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>5.03</v>
+        <v>2.3</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>09/09/25 17:32</t>
+          <t>09/10/25 09:03</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>77821</t>
+          <t>77873</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4690,17 +4698,17 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>ASICS Gel-NYC Cream Arctic Sky</t>
+          <t>Air Force 1 Rope Laces</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>40 EU - 7 US</t>
+          <t>38 EU - 5.5 US</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>1203A383-107</t>
+          <t>CW2288-111ME</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4721,17 +4729,17 @@
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>gestoriapradillo@gmail.com</t>
+          <t>kaaa-95@hotmail.com</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>LAURA</t>
+          <t>Karen</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>BORRAJO ROMERO</t>
+          <t>Serrano Sánchez</t>
         </is>
       </c>
       <c r="T30" t="inlineStr"/>
@@ -4747,24 +4755,16 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>an unknown source</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>cpc</t>
-        </is>
-      </c>
-      <c r="Z30" t="inlineStr">
-        <is>
-          <t>21366334315</t>
-        </is>
-      </c>
+          <t>webgains</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr"/>
@@ -4897,26 +4897,26 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Webravo SRL</t>
+          <t>Shoparize</t>
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>5.1</v>
+        <v>4.2</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>1.53</v>
+        <v>1.26</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>09/09/25 14:38</t>
+          <t>09/09/25 01:55</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>77790</t>
+          <t>77760</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4936,17 +4936,17 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Adidas SL 72 OG Maroon Preloved Brown</t>
+          <t>Adidas SL 72 RS Black Carbon</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>41.3 EU - 8 US</t>
+          <t>44 EU - 10 US</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>IE3425</t>
+          <t>JH5098</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -4967,20 +4967,24 @@
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>portella.marina@gmail.com</t>
+          <t>manuelopez.mlg@gmail.com</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Marina</t>
+          <t>Manuel</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Portella</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr"/>
+          <t>López Garrido</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>+34673369013</t>
+        </is>
+      </c>
       <c r="U32" t="inlineStr">
         <is>
           <t>First Order</t>
@@ -4993,10 +4997,14 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>direct</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr"/>
+          <t>an unknown source</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>webgains</t>
+        </is>
+      </c>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="inlineStr"/>
@@ -5006,26 +5014,26 @@
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>Shoparize</t>
+          <t>Webravo SRL</t>
         </is>
       </c>
       <c r="B33" s="16" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="C33" s="16" t="n">
-        <v>4.2</v>
+        <v>5.1</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>1.26</v>
+        <v>1.53</v>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>09/09/25 01:55</t>
+          <t>09/09/25 14:38</t>
         </is>
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>77760</t>
+          <t>77790</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr">
@@ -5045,17 +5053,17 @@
       </c>
       <c r="J33" s="15" t="inlineStr">
         <is>
-          <t>Adidas SL 72 RS Black Carbon</t>
+          <t>Adidas SL 72 OG Maroon Preloved Brown</t>
         </is>
       </c>
       <c r="K33" s="15" t="inlineStr">
         <is>
-          <t>44 EU - 10 US</t>
+          <t>41.3 EU - 8 US</t>
         </is>
       </c>
       <c r="L33" s="15" t="inlineStr">
         <is>
-          <t>JH5098</t>
+          <t>IE3425</t>
         </is>
       </c>
       <c r="M33" s="15" t="inlineStr">
@@ -5076,24 +5084,20 @@
       <c r="P33" s="15" t="inlineStr"/>
       <c r="Q33" s="15" t="inlineStr">
         <is>
-          <t>manuelopez.mlg@gmail.com</t>
+          <t>portella.marina@gmail.com</t>
         </is>
       </c>
       <c r="R33" s="15" t="inlineStr">
         <is>
-          <t>Manuel</t>
+          <t>Marina</t>
         </is>
       </c>
       <c r="S33" s="15" t="inlineStr">
         <is>
-          <t>López Garrido</t>
-        </is>
-      </c>
-      <c r="T33" s="15" t="inlineStr">
-        <is>
-          <t>+34673369013</t>
-        </is>
-      </c>
+          <t>Portella</t>
+        </is>
+      </c>
+      <c r="T33" s="15" t="inlineStr"/>
       <c r="U33" s="15" t="inlineStr">
         <is>
           <t>First Order</t>
@@ -5106,14 +5110,10 @@
       </c>
       <c r="W33" s="15" t="inlineStr">
         <is>
-          <t>an unknown source</t>
-        </is>
-      </c>
-      <c r="X33" s="15" t="inlineStr">
-        <is>
-          <t>webgains</t>
-        </is>
-      </c>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="X33" s="15" t="inlineStr"/>
       <c r="Y33" s="15" t="inlineStr"/>
       <c r="Z33" s="15" t="inlineStr"/>
       <c r="AA33" s="15" t="inlineStr"/>
@@ -5236,26 +5236,26 @@
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>LINKGAINS PTE.LTD.</t>
+          <t>LINKPREFER LIMITED</t>
         </is>
       </c>
       <c r="B35" s="16" t="n">
-        <v>90</v>
+        <v>280</v>
       </c>
       <c r="C35" s="16" t="n">
-        <v>5.4</v>
+        <v>16.8</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>1.62</v>
+        <v>5.04</v>
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>09/07/25 15:51</t>
+          <t>09/07/25 15:13</t>
         </is>
       </c>
       <c r="F35" s="15" t="inlineStr">
         <is>
-          <t>77615</t>
+          <t>77607</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr">
@@ -5275,17 +5275,17 @@
       </c>
       <c r="J35" s="15" t="inlineStr">
         <is>
-          <t>Puma Arizona Zebra</t>
+          <t>Adidas Gazelle Indoor Bad Bunny Cabo Rojo</t>
         </is>
       </c>
       <c r="K35" s="15" t="inlineStr">
         <is>
-          <t>37 EU - 5 US</t>
+          <t>38.6 EU - 6 US</t>
         </is>
       </c>
       <c r="L35" s="15" t="inlineStr">
         <is>
-          <t>404398-01</t>
+          <t>JS5052</t>
         </is>
       </c>
       <c r="M35" s="15" t="inlineStr">
@@ -5306,69 +5306,89 @@
       <c r="P35" s="15" t="inlineStr"/>
       <c r="Q35" s="15" t="inlineStr">
         <is>
-          <t>jessijuan2014@gmail.com</t>
+          <t>browses.owners-8u@icloud.com</t>
         </is>
       </c>
       <c r="R35" s="15" t="inlineStr">
         <is>
-          <t>Eva</t>
+          <t>Paula</t>
         </is>
       </c>
       <c r="S35" s="15" t="inlineStr">
         <is>
-          <t>Llopis</t>
+          <t>Schweitzer</t>
         </is>
       </c>
       <c r="T35" s="15" t="inlineStr">
         <is>
-          <t>+34650397617</t>
+          <t>+34680952342</t>
         </is>
       </c>
       <c r="U35" s="15" t="inlineStr">
         <is>
-          <t>Repeat Customer (Order #3)</t>
+          <t>First Order</t>
         </is>
       </c>
       <c r="V35" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W35" s="15" t="inlineStr">
         <is>
-          <t>direct</t>
-        </is>
-      </c>
-      <c r="X35" s="15" t="inlineStr"/>
-      <c r="Y35" s="15" t="inlineStr"/>
-      <c r="Z35" s="15" t="inlineStr"/>
-      <c r="AA35" s="15" t="inlineStr"/>
-      <c r="AB35" s="15" t="inlineStr"/>
+          <t>an unknown source</t>
+        </is>
+      </c>
+      <c r="X35" s="15" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="Y35" s="15" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="Z35" s="15" t="inlineStr">
+        <is>
+          <t>CAMPAÑA_ESCALADO_AD</t>
+        </is>
+      </c>
+      <c r="AA35" s="15" t="inlineStr">
+        <is>
+          <t>120206246202400135</t>
+        </is>
+      </c>
+      <c r="AB35" s="15" t="inlineStr">
+        <is>
+          <t>120231190735490135</t>
+        </is>
+      </c>
       <c r="AC35" s="15" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LINKPREFER LIMITED</t>
+          <t>LINKGAINS PTE.LTD.</t>
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>280</v>
+        <v>90</v>
       </c>
       <c r="C36" s="13" t="n">
-        <v>16.8</v>
+        <v>5.4</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>5.04</v>
+        <v>1.62</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>09/07/25 15:13</t>
+          <t>09/07/25 15:51</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>77607</t>
+          <t>77615</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5388,17 +5408,17 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Adidas Gazelle Indoor Bad Bunny Cabo Rojo</t>
+          <t>Puma Arizona Zebra</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>38.6 EU - 6 US</t>
+          <t>37 EU - 5 US</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>JS5052</t>
+          <t>404398-01</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -5419,64 +5439,44 @@
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>browses.owners-8u@icloud.com</t>
+          <t>jessijuan2014@gmail.com</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Paula</t>
+          <t>Eva</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Schweitzer</t>
+          <t>Llopis</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>+34680952342</t>
+          <t>+34650397617</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>First Order</t>
+          <t>Repeat Customer (Order #3)</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>an unknown source</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t>CAMPAÑA_ESCALADO_AD</t>
-        </is>
-      </c>
-      <c r="AA36" t="inlineStr">
-        <is>
-          <t>120206246202400135</t>
-        </is>
-      </c>
-      <c r="AB36" t="inlineStr">
-        <is>
-          <t>120231190735490135</t>
-        </is>
-      </c>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -5817,7 +5817,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Purplee Corp</t>
         </is>
       </c>
       <c r="B40" s="13" t="n">
@@ -5831,12 +5831,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>09/05/25 20:13</t>
+          <t>09/02/25 21:53</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>77431</t>
+          <t>6870936355157</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>43 EU - 10 US</t>
+          <t>41 EU - 8.5 US</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -5887,22 +5887,22 @@
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>pj_sanchez17@yahoo.es</t>
+          <t>sandrafresita@live.com</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Paula</t>
+          <t>Christian</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Sanchez fernandez</t>
+          <t>Sáez badia</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>+34655472907</t>
+          <t>+34660229457</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -5917,7 +5917,7 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="X40" t="inlineStr"/>
@@ -5930,26 +5930,26 @@
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>Purplee Corp</t>
+          <t>Invoke AB</t>
         </is>
       </c>
       <c r="B41" s="16" t="n">
-        <v>120</v>
+        <v>320</v>
       </c>
       <c r="C41" s="16" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>1.8</v>
+        <v>4.8</v>
       </c>
       <c r="E41" s="15" t="inlineStr">
         <is>
-          <t>09/02/25 21:53</t>
+          <t>09/04/25 19:12</t>
         </is>
       </c>
       <c r="F41" s="15" t="inlineStr">
         <is>
-          <t>6870936355157</t>
+          <t>77301</t>
         </is>
       </c>
       <c r="G41" s="15" t="inlineStr">
@@ -5969,17 +5969,17 @@
       </c>
       <c r="J41" s="15" t="inlineStr">
         <is>
-          <t>Puma LaMelo Ball LaFrancé Amour Moment</t>
+          <t>Air Jordan 3 Retro Black Cat</t>
         </is>
       </c>
       <c r="K41" s="15" t="inlineStr">
         <is>
-          <t>41 EU - 8.5 US</t>
+          <t>41 EU - 8 US</t>
         </is>
       </c>
       <c r="L41" s="15" t="inlineStr">
         <is>
-          <t>310864-01</t>
+          <t>CT8532-001</t>
         </is>
       </c>
       <c r="M41" s="15" t="inlineStr">
@@ -6000,22 +6000,22 @@
       <c r="P41" s="15" t="inlineStr"/>
       <c r="Q41" s="15" t="inlineStr">
         <is>
-          <t>sandrafresita@live.com</t>
+          <t>alexitomendo1960@gmail.com</t>
         </is>
       </c>
       <c r="R41" s="15" t="inlineStr">
         <is>
-          <t>Christian</t>
+          <t>Alexander</t>
         </is>
       </c>
       <c r="S41" s="15" t="inlineStr">
         <is>
-          <t>Sáez badia</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="T41" s="15" t="inlineStr">
         <is>
-          <t>+34660229457</t>
+          <t>+34634868685</t>
         </is>
       </c>
       <c r="U41" s="15" t="inlineStr">
@@ -6030,10 +6030,14 @@
       </c>
       <c r="W41" s="15" t="inlineStr">
         <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="X41" s="15" t="inlineStr"/>
+          <t>an unknown source</t>
+        </is>
+      </c>
+      <c r="X41" s="15" t="inlineStr">
+        <is>
+          <t>webgains</t>
+        </is>
+      </c>
       <c r="Y41" s="15" t="inlineStr"/>
       <c r="Z41" s="15" t="inlineStr"/>
       <c r="AA41" s="15" t="inlineStr"/>
@@ -6043,26 +6047,26 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Invoke AB</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>320</v>
+        <v>120</v>
       </c>
       <c r="C42" s="13" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>4.8</v>
+        <v>1.8</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>09/04/25 19:12</t>
+          <t>09/05/25 20:13</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>77301</t>
+          <t>77431</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -6082,17 +6086,17 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Air Jordan 3 Retro Black Cat</t>
+          <t>Puma LaMelo Ball LaFrancé Amour Moment</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>41 EU - 8 US</t>
+          <t>43 EU - 10 US</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>CT8532-001</t>
+          <t>310864-01</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -6113,22 +6117,22 @@
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>alexitomendo1960@gmail.com</t>
+          <t>pj_sanchez17@yahoo.es</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Alexander</t>
+          <t>Paula</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Sanchez fernandez</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>+34634868685</t>
+          <t>+34655472907</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -6143,14 +6147,10 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>an unknown source</t>
-        </is>
-      </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>webgains</t>
-        </is>
-      </c>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr"/>
       <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
@@ -6160,56 +6160,56 @@
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Skimbit LTD</t>
         </is>
       </c>
       <c r="B43" s="16" t="n">
-        <v>250</v>
+        <v>96</v>
       </c>
       <c r="C43" s="16" t="n">
-        <v>15</v>
+        <v>4.8</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>4.5</v>
+        <v>1.44</v>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>09/04/25 16:31</t>
+          <t>09/02/25 15:23</t>
         </is>
       </c>
       <c r="F43" s="15" t="inlineStr">
         <is>
-          <t>77278</t>
+          <t>77081</t>
         </is>
       </c>
       <c r="G43" s="15" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="H43" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="J43" s="15" t="inlineStr">
         <is>
-          <t>Air Jordan 3 Retro Pure Money</t>
+          <t>Adidas Campus 00s Grey White</t>
         </is>
       </c>
       <c r="K43" s="15" t="inlineStr">
         <is>
-          <t>41 EU - 8 US</t>
+          <t>42 EU - 8.5 US</t>
         </is>
       </c>
       <c r="L43" s="15" t="inlineStr">
         <is>
-          <t>CT8532-111</t>
+          <t>HQ8707</t>
         </is>
       </c>
       <c r="M43" s="15" t="inlineStr">
@@ -6230,40 +6230,44 @@
       <c r="P43" s="15" t="inlineStr"/>
       <c r="Q43" s="15" t="inlineStr">
         <is>
-          <t>sebastiancalvovinasco076@gmail.com</t>
+          <t>noapataly1602@gmail.com</t>
         </is>
       </c>
       <c r="R43" s="15" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Patricia</t>
         </is>
       </c>
       <c r="S43" s="15" t="inlineStr">
         <is>
-          <t>Calvo vinasco</t>
+          <t>Da Silva</t>
         </is>
       </c>
       <c r="T43" s="15" t="inlineStr">
         <is>
-          <t>+34655364031</t>
+          <t>+32490401121</t>
         </is>
       </c>
       <c r="U43" s="15" t="inlineStr">
         <is>
-          <t>Repeat Customer (Order #2)</t>
+          <t>First Order</t>
         </is>
       </c>
       <c r="V43" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W43" s="15" t="inlineStr">
         <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="X43" s="15" t="inlineStr"/>
+          <t>an unknown source</t>
+        </is>
+      </c>
+      <c r="X43" s="15" t="inlineStr">
+        <is>
+          <t>chatgpt.com</t>
+        </is>
+      </c>
       <c r="Y43" s="15" t="inlineStr"/>
       <c r="Z43" s="15" t="inlineStr"/>
       <c r="AA43" s="15" t="inlineStr"/>
@@ -6273,56 +6277,56 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Skimbit LTD</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>96</v>
+        <v>250</v>
       </c>
       <c r="C44" s="13" t="n">
-        <v>4.8</v>
+        <v>15</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>1.44</v>
+        <v>4.5</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>09/02/25 15:23</t>
+          <t>09/04/25 16:31</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>77081</t>
+          <t>77278</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I44" s="14" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Adidas Campus 00s Grey White</t>
+          <t>Air Jordan 3 Retro Pure Money</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>42 EU - 8.5 US</t>
+          <t>41 EU - 8 US</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>HQ8707</t>
+          <t>CT8532-111</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -6343,44 +6347,40 @@
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>noapataly1602@gmail.com</t>
+          <t>sebastiancalvovinasco076@gmail.com</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Patricia</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Da Silva</t>
+          <t>Calvo vinasco</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>+32490401121</t>
+          <t>+34655364031</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>First Order</t>
+          <t>Repeat Customer (Order #2)</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>an unknown source</t>
-        </is>
-      </c>
-      <c r="X44" t="inlineStr">
-        <is>
-          <t>chatgpt.com</t>
-        </is>
-      </c>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr"/>
       <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="inlineStr"/>
@@ -6708,22 +6708,22 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>127.5</v>
+        <v>70</v>
       </c>
       <c r="C2" s="13" t="n">
-        <v>7.65</v>
+        <v>4.2</v>
       </c>
       <c r="D2" s="13" t="n">
-        <v>2.3</v>
+        <v>1.26</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>09/30/25 16:25</t>
+          <t>09/30/25 12:49</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>79375</t>
+          <t>79361</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6745,26 +6745,26 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Digital Expand</t>
+          <t>Mathias Kraft</t>
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>4.2</v>
+        <v>10.8</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>1.26</v>
+        <v>3.24</v>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>09/30/25 12:49</t>
+          <t>09/30/25 15:30</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>79361</t>
+          <t>79365</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
@@ -6786,26 +6786,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mathias Kraft</t>
+          <t>Digital Expand</t>
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>180</v>
+        <v>127.5</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>10.8</v>
+        <v>7.65</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>3.24</v>
+        <v>2.3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>09/30/25 15:30</t>
+          <t>09/30/25 16:25</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>79365</t>
+          <t>79375</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6950,31 +6950,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Webravo SRL</t>
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>330</v>
+        <v>110</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>19.8</v>
+        <v>6.6</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>5.94</v>
+        <v>1.98</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>09/24/25 14:24</t>
+          <t>09/22/25 20:03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>78891</t>
+          <t>78812</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -7073,31 +7073,31 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Webravo SRL</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>110</v>
+        <v>330</v>
       </c>
       <c r="C11" s="16" t="n">
-        <v>6.6</v>
+        <v>19.8</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>1.98</v>
+        <v>5.94</v>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>09/22/25 20:03</t>
+          <t>09/24/25 14:24</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>78812</t>
+          <t>78891</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -7114,26 +7114,26 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Purplee Corp</t>
+          <t>Invoke AB</t>
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>170</v>
+        <v>350</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>10.2</v>
+        <v>21</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>3.06</v>
+        <v>6.3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>09/22/25 14:45</t>
+          <t>09/20/25 11:34</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6903116824917</t>
+          <t>6900010221909</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -7155,26 +7155,26 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Digital Expand</t>
+          <t>Purplee Corp</t>
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>6</v>
+        <v>10.2</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>1.8</v>
+        <v>3.06</v>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>09/18/25 19:39</t>
+          <t>09/22/25 14:45</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>6897694179669</t>
+          <t>6903116824917</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -7184,38 +7184,38 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Invoke AB</t>
+          <t>Digital Expand</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>350</v>
+        <v>120</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>6.3</v>
+        <v>1.8</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>09/20/25 11:34</t>
+          <t>09/18/25 19:39</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>6900010221909</t>
+          <t>6897694179669</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -7225,38 +7225,38 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Pashion.dk ApS</t>
         </is>
       </c>
       <c r="B15" s="16" t="n">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="C15" s="16" t="n">
-        <v>6.6</v>
+        <v>14</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>1.98</v>
+        <v>4.2</v>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>09/19/25 23:39</t>
+          <t>09/16/25 20:51</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>78602</t>
+          <t>6894848966997</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
@@ -7266,38 +7266,38 @@
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Webravo SRL</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1.62</v>
+        <v>1.98</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>09/20/25 11:53</t>
+          <t>09/19/25 23:39</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>78608</t>
+          <t>78602</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -7319,26 +7319,26 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Pashion.dk ApS</t>
+          <t>Webravo SRL</t>
         </is>
       </c>
       <c r="B17" s="16" t="n">
-        <v>280</v>
+        <v>90</v>
       </c>
       <c r="C17" s="16" t="n">
-        <v>14</v>
+        <v>5.4</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>4.2</v>
+        <v>1.62</v>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>09/16/25 20:51</t>
+          <t>09/20/25 11:53</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>6894848966997</t>
+          <t>78608</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -7348,12 +7348,12 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
     </row>
@@ -7401,26 +7401,26 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Pashion.dk ApS</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B19" s="16" t="n">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="C19" s="16" t="n">
-        <v>6</v>
+        <v>5.28</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>1.8</v>
+        <v>1.58</v>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>09/16/25 16:05</t>
+          <t>09/15/25 11:50</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>78437</t>
+          <t>78383</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
@@ -7430,12 +7430,12 @@
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I19" s="17" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
     </row>
@@ -7483,26 +7483,26 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Pashion.dk ApS</t>
         </is>
       </c>
       <c r="B21" s="16" t="n">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="C21" s="16" t="n">
-        <v>5.28</v>
+        <v>6</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>1.58</v>
+        <v>1.8</v>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>09/15/25 11:50</t>
+          <t>09/16/25 16:05</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>78383</t>
+          <t>78437</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
@@ -7512,38 +7512,38 @@
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pashion.dk ApS</t>
+          <t>Purplee Corp</t>
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>120</v>
+        <v>82.5</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>6</v>
+        <v>4.95</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>1.8</v>
+        <v>1.49</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>09/15/25 11:46</t>
+          <t>09/14/25 12:50</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>78382</t>
+          <t>6891134681429</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7553,38 +7553,38 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Pashion.dk ApS</t>
         </is>
       </c>
       <c r="B23" s="16" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="C23" s="16" t="n">
-        <v>5.76</v>
+        <v>6</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>1.73</v>
+        <v>1.8</v>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>09/14/25 22:07</t>
+          <t>09/15/25 11:46</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>78374</t>
+          <t>78382</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
@@ -7594,38 +7594,38 @@
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Purplee Corp</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>82.5</v>
+        <v>96</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>4.95</v>
+        <v>5.76</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>1.49</v>
+        <v>1.73</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>09/14/25 12:50</t>
+          <t>09/14/25 22:07</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>6891134681429</t>
+          <t>78374</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7647,26 +7647,26 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Digital Expand</t>
         </is>
       </c>
       <c r="B25" s="16" t="n">
-        <v>750</v>
+        <v>550</v>
       </c>
       <c r="C25" s="16" t="n">
-        <v>37.5</v>
+        <v>27.5</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>11.25</v>
+        <v>8.25</v>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>09/13/25 10:43</t>
+          <t>09/11/25 16:14</t>
         </is>
       </c>
       <c r="F25" s="15" t="inlineStr">
         <is>
-          <t>78157</t>
+          <t>6887025475925</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">
@@ -7688,26 +7688,26 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Digital Expand</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>550</v>
+        <v>750</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>27.5</v>
+        <v>37.5</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>8.25</v>
+        <v>11.25</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>09/11/25 16:14</t>
+          <t>09/13/25 10:43</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>6887025475925</t>
+          <t>78157</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7811,26 +7811,26 @@
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>Klarna Bank AB UK Branch</t>
+          <t>LINKGAINS PTE.LTD.</t>
         </is>
       </c>
       <c r="B29" s="16" t="n">
-        <v>153</v>
+        <v>335</v>
       </c>
       <c r="C29" s="16" t="n">
-        <v>7.65</v>
+        <v>16.75</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>2.3</v>
+        <v>5.03</v>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>09/10/25 09:03</t>
+          <t>09/09/25 17:32</t>
         </is>
       </c>
       <c r="F29" s="15" t="inlineStr">
         <is>
-          <t>77873</t>
+          <t>77821</t>
         </is>
       </c>
       <c r="G29" s="15" t="inlineStr">
@@ -7852,26 +7852,26 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LINKGAINS PTE.LTD.</t>
+          <t>Klarna Bank AB UK Branch</t>
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>335</v>
+        <v>153</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>16.75</v>
+        <v>7.65</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>5.03</v>
+        <v>2.3</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>09/09/25 17:32</t>
+          <t>09/10/25 09:03</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>77821</t>
+          <t>77873</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7934,26 +7934,26 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Webravo SRL</t>
+          <t>Shoparize</t>
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>5.1</v>
+        <v>4.2</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>1.53</v>
+        <v>1.26</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>09/09/25 14:38</t>
+          <t>09/09/25 01:55</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>77790</t>
+          <t>77760</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7975,26 +7975,26 @@
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>Shoparize</t>
+          <t>Webravo SRL</t>
         </is>
       </c>
       <c r="B33" s="16" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="C33" s="16" t="n">
-        <v>4.2</v>
+        <v>5.1</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>1.26</v>
+        <v>1.53</v>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>09/09/25 01:55</t>
+          <t>09/09/25 14:38</t>
         </is>
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>77760</t>
+          <t>77790</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr">
@@ -8057,26 +8057,26 @@
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>LINKGAINS PTE.LTD.</t>
+          <t>LINKPREFER LIMITED</t>
         </is>
       </c>
       <c r="B35" s="16" t="n">
-        <v>90</v>
+        <v>280</v>
       </c>
       <c r="C35" s="16" t="n">
-        <v>5.4</v>
+        <v>16.8</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>1.62</v>
+        <v>5.04</v>
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>09/07/25 15:51</t>
+          <t>09/07/25 15:13</t>
         </is>
       </c>
       <c r="F35" s="15" t="inlineStr">
         <is>
-          <t>77615</t>
+          <t>77607</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr">
@@ -8098,26 +8098,26 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LINKPREFER LIMITED</t>
+          <t>LINKGAINS PTE.LTD.</t>
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>280</v>
+        <v>90</v>
       </c>
       <c r="C36" s="13" t="n">
-        <v>16.8</v>
+        <v>5.4</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>5.04</v>
+        <v>1.62</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>09/07/25 15:13</t>
+          <t>09/07/25 15:51</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>77607</t>
+          <t>77615</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8262,7 +8262,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Purplee Corp</t>
         </is>
       </c>
       <c r="B40" s="13" t="n">
@@ -8276,12 +8276,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>09/05/25 20:13</t>
+          <t>09/02/25 21:53</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>77431</t>
+          <t>6870936355157</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8303,26 +8303,26 @@
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>Purplee Corp</t>
+          <t>Invoke AB</t>
         </is>
       </c>
       <c r="B41" s="16" t="n">
-        <v>120</v>
+        <v>320</v>
       </c>
       <c r="C41" s="16" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>1.8</v>
+        <v>4.8</v>
       </c>
       <c r="E41" s="15" t="inlineStr">
         <is>
-          <t>09/02/25 21:53</t>
+          <t>09/04/25 19:12</t>
         </is>
       </c>
       <c r="F41" s="15" t="inlineStr">
         <is>
-          <t>6870936355157</t>
+          <t>77301</t>
         </is>
       </c>
       <c r="G41" s="15" t="inlineStr">
@@ -8344,26 +8344,26 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Invoke AB</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>320</v>
+        <v>120</v>
       </c>
       <c r="C42" s="13" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>4.8</v>
+        <v>1.8</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>09/04/25 19:12</t>
+          <t>09/05/25 20:13</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>77301</t>
+          <t>77431</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8385,82 +8385,82 @@
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>BlueVision Interactive Limited</t>
+          <t>Skimbit LTD</t>
         </is>
       </c>
       <c r="B43" s="16" t="n">
-        <v>250</v>
+        <v>96</v>
       </c>
       <c r="C43" s="16" t="n">
-        <v>15</v>
+        <v>4.8</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>4.5</v>
+        <v>1.44</v>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>09/04/25 16:31</t>
+          <t>09/02/25 15:23</t>
         </is>
       </c>
       <c r="F43" s="15" t="inlineStr">
         <is>
-          <t>77278</t>
+          <t>77081</t>
         </is>
       </c>
       <c r="G43" s="15" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="H43" s="15" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Reventa</t>
         </is>
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Skimbit LTD</t>
+          <t>BlueVision Interactive Limited</t>
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>96</v>
+        <v>250</v>
       </c>
       <c r="C44" s="13" t="n">
-        <v>4.8</v>
+        <v>15</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>1.44</v>
+        <v>4.5</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>09/02/25 15:23</t>
+          <t>09/04/25 16:31</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>77081</t>
+          <t>77278</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Reventa</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="I44" s="14" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
     </row>

</xml_diff>